<commit_message>
Update Mooc.md with Matterport integration details and restructure course content
</commit_message>
<xml_diff>
--- a/Files/S3_MOOC_Template_Grupo1.xlsx
+++ b/Files/S3_MOOC_Template_Grupo1.xlsx
@@ -646,7 +646,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1" s="5">
+    <row r="10" ht="90" customHeight="1" s="5">
       <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Matterport</t>
@@ -654,7 +654,7 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>A definir (espaço e forma de integração).</t>
+          <t>Casa real digitalizada em 3D (a «casa da D. Rosa e da Ana», capturada pelo grupo com a app Matterport Capture) como fio condutor das 5 lições + espaço de acolhimento encenado numa sala da escola para a L4 (plano B: espaço público do Matterport Discover). Tags em 2 cores: azul = pessoa com demência, laranja = cuidador. Na Udemy: 1-2 min de vídeo gravado da visita em cada lição + link «Visita 3D» nos recursos (opcional, nunca obrigatório para o quiz). Espaços «não listados», 1 por conta grátis; consentimento do proprietário e remoção de dados pessoais antes da captura.</t>
         </is>
       </c>
     </row>
@@ -685,8 +685,8 @@
     <col width="36.109375" customWidth="1" style="5" min="11" max="11"/>
     <col width="41.6640625" customWidth="1" style="5" min="12" max="12"/>
     <col width="29.88671875" customWidth="1" style="5" min="13" max="13"/>
-    <col width="48.33203125" customWidth="1" style="5" min="14" max="14"/>
-    <col width="36.109375" customWidth="1" style="5" min="15" max="15"/>
+    <col width="52" customWidth="1" style="5" min="14" max="14"/>
+    <col width="60" customWidth="1" style="5" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="72" customHeight="1" s="5">
@@ -853,13 +853,16 @@
       <c r="N2" s="19" t="inlineStr">
         <is>
           <t>Quiz: associar cenário de crise → impacto na pessoa com demência (4 perguntas).
-Reflexão: «O que dá segurança à pessoa de quem cuida?» (registo pessoal).</t>
+Reflexão: «O que dá segurança à pessoa de quem cuida?» (registo pessoal).
+Visita 3D (opcional): «Encontre 3 coisas na casa que dão segurança à pessoa».</t>
         </is>
       </c>
       <c r="O2" s="19" t="inlineStr">
         <is>
           <t>Responsável: Bruno Lopes
-Integração Matterport: a definir.</t>
+Integração Matterport: Espaço: casa da D. Rosa.
+Visita guiada «A casa pelos olhos da D. Rosa»: tags azuis nas âncoras de segurança (cadeira habitual, fotografias, relógio, cozinha); tag laranja «E a Ana? Onde descansa?».
+Vídeo: a mesma divisão com o que a crise traz (ruído, luzes, malas no corredor).</t>
         </is>
       </c>
     </row>
@@ -936,13 +939,16 @@
         <is>
           <t>Atividade: completar o kit (escolher os itens certos de uma lista com distratores).
 Descarregar e preencher a ficha da pessoa e o plano de apoio.
-Quiz (4 perguntas).</t>
+Quiz (4 perguntas).
+Visita 3D (opcional): percorrer a casa e compor a lista do kit antes de ver a checklist.</t>
         </is>
       </c>
       <c r="O3" s="19" t="inlineStr">
         <is>
           <t>Responsável: Tiago Teixeira
-Integração Matterport: a definir.</t>
+Integração Matterport: Espaço: casa da D. Rosa.
+«Caça ao kit»: tags azuis onde estão os itens (medicação e receitas, documentos, fotografia, óculos, objeto de conforto); kit junto à porta; ficha da pessoa no frigorífico (tag com link para o PDF); medir o corredor até à saída.
+Tag laranja no telefone: rede de 3 contactos e substituto.</t>
         </is>
       </c>
     </row>
@@ -1016,13 +1022,16 @@
       <c r="N4" s="19" t="inlineStr">
         <is>
           <t>Quiz de cenários: «O que dizias/fazias?» com feedback em cada opção (4 situações).
-Exercício: praticar a técnica de respiração guiada (1 min).</t>
+Exercício: praticar a técnica de respiração guiada (1 min).
+Visita 3D (opcional): «Para onde levaria a D. Rosa e o que desligaria?» (resposta no quiz).</t>
         </is>
       </c>
       <c r="O4" s="19" t="inlineStr">
         <is>
           <t>Responsável: Rodrigo Silva
-Integração Matterport: a definir.</t>
+Integração Matterport: Espaço: casa da D. Rosa (sala da cena).
+«Reduzir estímulos»: tags azuis nas fontes de estímulo (TV/rádio, janela, espelho, porta da rua) e no «canto calmo»; tag com o vídeo da dramatização (YouTube não listado) no sítio da cena.
+Tag laranja «Pausa de 10 segundos» à porta da sala.</t>
         </is>
       </c>
     </row>
@@ -1098,13 +1107,16 @@
       <c r="N5" s="19" t="inlineStr">
         <is>
           <t>Quiz de decisão: ordenar prioridades e escolher quando encaminhar (4 perguntas).
-Descarregar o cartão de bolso com sinais de alarme e contactos.</t>
+Descarregar o cartão de bolso com sinais de alarme e contactos.
+Visita 3D (opcional): «Escolha o melhor lugar para a D. Rosa ficar» (quiz com feedback por opção).</t>
         </is>
       </c>
       <c r="O5" s="19" t="inlineStr">
         <is>
           <t>Responsável: Ricardo Ferreira
-Integração Matterport: a definir.</t>
+Integração Matterport: Espaço: acolhimento encenado (sala da escola; plano B: Discover ou só a casa).
+Visita antes de chegar: tags no balcão de registo (sinalizar a demência), zona de descanso, casa de banho e saídas; tags com sinais de alarme, 112 / SNS 24 e cartão de bolso (PDF).
+Se for só a casa: decisão «ficar ou sair».</t>
         </is>
       </c>
     </row>
@@ -1181,13 +1193,16 @@
         <is>
           <t>Autoavaliação de sobrecarga (escala simples).
 Quiz final do curso (6 perguntas, cobre as 5 lições).
-Plano pessoal: «3 apoios a que posso recorrer».</t>
+Plano pessoal: «3 apoios a que posso recorrer».
+Visita 3D (opcional): percorrer a casa e identificar 1 ação por lição (síntese do curso).
+Exercício para casa: aplicar a mesma checklist à sua própria casa.</t>
         </is>
       </c>
       <c r="O6" s="19" t="inlineStr">
         <is>
           <t>Responsável: Evandro Carvalho
-Integração Matterport: a definir.</t>
+Integração Matterport: Espaço: casa da D. Rosa.
+«Regresso a casa»: tags azuis de «repor» (kit reposto, rotina, objetos no sítio, calendário à vista); tags laranja com descanso do cuidador e apoios (SNS 24, Alzheimer Portugal, Estatuto do Cuidador Informal) com links.</t>
         </is>
       </c>
     </row>

</xml_diff>